<commit_message>
feat: update Firm-3 invoice processing and enhance error logging
</commit_message>
<xml_diff>
--- a/TallyCodes/invoice/Log/invoice_sync_logs.xlsx
+++ b/TallyCodes/invoice/Log/invoice_sync_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K12"/>
+  <dimension ref="A2:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -917,10 +917,433 @@
           <t>CFB PIXIE LIQUID BLUE 100 ML-71000120 - V PLATE: rate missing or zero | CFB PIXIE LIQUID BLUE 100 ML-71000120 - V PLATE: amount missing or zero</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:06:07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>87172914-2d61-456b-ac49-dc228b7822e0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LNKI/INV/26-27/00001</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NATCO PHARMA LIMITED</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Posted successfully to Tally</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>LNKI/INV/26-27/00001</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>6886</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:43:53</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FAILURE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PRECHECK</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>733ae812-c44c-48e8-a5cb-c01f8b89a095</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LNCB-2/26-27/00001</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>LAXMI NARAYAN KRAFT INDUSTRIES</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Tally is unavailable on http://127.0.0.1:9002: HTTPConnectionPool(host='127.0.0.1', port=9002): Max retries exceeded with url: / (Caused by NewConnectionError("HTTPConnection(host='127.0.0.1', port=9002): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it"))</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:45:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FAILURE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PRECHECK</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>17df4cac-4ebc-48ca-ab34-ea5087546383</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LNCB-2/INV/26-27/00003</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UNITED SPIRITS LIMITED</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Stock Item 'OC-MCDLUXTTN-BLD-G180- 8.64-WP2P-KT3P7V13' not found in Tally response. Debug XML: d:\LNGRP\TallyCodes\invoice\Log\tally_debug\stock_item_missing_node_20261016_164538_OC-MCDLUXTTN-BLD-G180-_8.64-WP2P-KT3P7V13.xml</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:45:39</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>733ae812-c44c-48e8-a5cb-c01f8b89a095</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LNCB-2/26-27/00001</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>LAXMI NARAYAN KRAFT INDUSTRIES</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Posted successfully to Tally</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>LNCB-2/26-27/00001</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>48188</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:45:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>7435be59-e911-4869-a327-575a5f74fa25</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LNCB-2/26-27/00002</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>LAXMI NARAYAN KRAFT INDUSTRIES</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Posted successfully to Tally</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>LNCB-2/26-27/00002</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>48189</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:24:32</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4a184270-204b-4772-bf76-29256ea95078</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LNCB-1/26-27/00001</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Laxmi Narayan Corrugated Boards LLP (Unit-II)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Posted successfully to Tally</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>LNCB-1/26-27/00001</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>138412</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:24:33</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>b3a3fb63-197d-433f-b382-c16c0b447ce9</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LNCB-1/26-27/00002</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Laxmi Narayan Corrugated Boards LLP (Unit-II)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Posted successfully to Tally</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>LNCB-1/26-27/00002</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>138413</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:24:34</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>68b4fc3d-3f10-4c61-8bf6-009a191193e5</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LNCB-1/26-27/00003</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Laxmi Narayan Corrugated Boards LLP (Unit-II)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Posted successfully to Tally</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>LNCB-1/26-27/00003</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>138414</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>d:\LNGRP\TallyCodes\invoice\invFirm1.py</t>
         </is>

</xml_diff>